<commit_message>
Reorg T0.0: reconcile overlap audit vs HEAD (9 findings re-verified, col M added)
- 2 partially addressed: control-drain-1 (V189 net-value gate kills the worst
  boundary; net-0 fall-through survives), shields-response-2 (ee0a1b435 unified
  2 of 3 occupation predicates; ShieldStrategy trigger-A copy remains).
- 7 still valid at HEAD: control-drain-5 + deploy-sequencing-1 remain HIGH;
  control-drain-4 WIDENED (V189 protections live in the evaluator brain only).
- 41 non-refuted rows verified untouched by diff-hunk check vs base 8392f3868.
- Handoff §11 baton updated. No src/ changes this step.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/Rando_Overlap_Audit_2026-07-04.xlsx
+++ b/resources/Rando_Overlap_Audit_2026-07-04.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,16 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -107,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -129,6 +139,21 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -509,6 +534,7 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,6 +598,11 @@
           <t>Evidence (file:line)</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Status @HEAD (T0.0 reconcile 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="147" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -634,6 +665,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/BattleEvaluator.java:396-419 (draw estimate 399-409, no ability filter despite comment 397), :186 (abilityDiff*2.5), :429-434 (-800); ActionTextEvaluator.java:4032 (abilityDiff*2.5), :4050-4051 (+120); BattlePredictor.java:31-58 (winRate model, 1 destiny 0-6 per draw)</t>
         </is>
       </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="147" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -696,6 +732,11 @@
           <t>ActionTextEvaluator.java:5309 (V48 -50 via VERY_BAD_DELTA, no return), :5324-5368 (V52 FIX 14 +300/+200/+100 tiers), :5375-5399 (V29.9 +30/+40), constants :29-32 (VERY_BAD_DELTA=-50); reachability: BO branch entered at :5167, V140 waiver return :5272 not taken, V104 only fires for drain&lt;=1 at :5284</t>
         </is>
       </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>PARTIALLY-ADDRESSED (sev now low) by 88b5170de, cb98f0075 — V189 (88f5.., refined by cb98f0075) now runs upstream of the whole V48/FIX-14 region: it queries the engine's getInitiateForceDrainCost, flat-blocks net &lt;= -2 drains (-2000 + return) and budget-gates net -1 drains against forcePile - cost &gt;= plannedHandDeploys + 2, returning before FIX 14/V29.9 can score. The finding's exact boundary (turn 1, drain 2, cost 3, force 6, deploy 3) is blocked: 6-3=3 &lt; 3+2. The V140 false</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="147" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -758,6 +799,11 @@
           <t>ActionTextEvaluator.java:5094-5101 (V25 static icon check), :5218-5225 (V140 modifiersQuerying.isBattleground on the same gameState in the same method), :5118-5123 (V25 -9999 block gated on the static check)</t>
         </is>
       </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now high) — The V25 Simple Tricks block is byte-identical to the audited version; git -L shows no post-audit commit touched lines 5159-5204 (last change was pre-audit snapshot 351a0523b). It still derives battleground status from static printed icons, so a dual-icon site made non-battleground by dynamic modification still slips past the -9999 block and Rando drains into a guaranteed Simple Tricks cancel; the upstream V189 net-va</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="147" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -820,6 +866,11 @@
           <t>ActionTextEvaluator.java:107 (blocked check), :126-149 (V169 endangered check + -400), :152-155 (hard veto -100000 + continue); MoveEvaluator.java:151-196 (blocked gate; soft path ctor -400 + addReasoning -400 at :191-192, continue at :195), :197-200 (hard path -9999 doubled to -19998), :54-57 (VERY_GOOD_DELTA=150, GOOD_DELTA=10), :1687-1694 + :1777-1780 (retreat/flee bonuses unreachable after continue); EvaluatedAction.java:27-44 + :63-67 (ctor score + reasoning delta + merge all add); CombinedEvaluator.java:71-86 (merge); ActionTextEvaluator.java:3505-3548 (V35.4 +150/+250); PassEvaluator.java:85 (Pass base 5)</t>
         </is>
       </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="147" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -882,6 +933,11 @@
           <t>PassEvaluator.java:33-57 (canEvaluate); CombinedEvaluator.java:20 (BAD_ACTION_THRESHOLD -100), :190-232 (V148 canPass at :206-213, dead duplicate condition at :226); DecisionSafety.java:59-120 (mustChoose V148 carve at :66-84); PassEvaluator.java:85-171 (Pass +5..+60 when it does run)</t>
         </is>
       </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="147" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -944,6 +1000,11 @@
           <t>ActionTextEvaluator.java:4227-4258 (V82 block runs first, unconditional, +2500 at 4243-4246); ActionTextEvaluator.java:4260-4276 (hardBlocked initialized AFTER V82; Guard 1 reserve&lt;=2 adds only -400 at 4269); ActionTextEvaluator.java:4492-4499 (baseline/V67ai gated on !hardBlocked — V82 is not); ActionTextEvaluator.java:341-343 (V116 +100 floor, earlier in method); ActionTextEvaluator.java:1148-1151 (V100 +1500, earlier in method); DeployEvaluator.java:531-534 (DeployEvaluator only processes actions containing 'deploy', so its own -9999 counterpart never runs for 'take ... into hand' phrasings)</t>
         </is>
       </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now high) — None of the six post-audit commits touched the mechanism: fcec408b9 changed only the V177 category-rescue block (~line 261-293), 88b5170de/cb98f0075 changed only the drain region (~5074+), and the other three didn't touch ActionTextEvaluator. At HEAD the V82 +2500 site-pull bonus still fires before hardBlocked exists, Guard 1 (reserve&lt;=2) still adds only -400, and hardBlocked still suppresses only the V60 baseline/V6</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="147" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1006,6 +1067,11 @@
           <t>DeployEvaluator.java:3416-3446 (V67ai tier switch, 2000/1800/1600/1500, fed by V67i detection at 3344-3414); ActionTextEvaluator.java:4662-4709 (identical V67ai tier switch at 4697-4703, fed by V67l detection at 4508-4549); CombinedEvaluator.java:74-82 (same actionId scores merged additively); ActionTextEvaluator.java:4653-4661 (V131 downgrade -2000, comment says 'neutralize V67ai's bonus (max +2000)'); DeployEvaluator.java:526-534,558-562 (DeployEvaluator scores any action containing 'deploy', base +50)</t>
         </is>
       </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="147" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1068,6 +1134,11 @@
           <t>DeployPhaseScript.java:224-231 (into-hand pulls excluded from all steps); CombinedEvaluator.java:109-148 (walk picks only from buckets; buckets exhausted -&gt; PASS at 139-148, never re-scans non-bucket actions); RandoCalAi.java:1130-1144 (DPS applied to every CARD_ACTION_CHOICE during DEPLOY); ActionTextEvaluator.java:4190-4204,4492-4499 (V60 scores into-hand pulls +150); ActionTextEvaluator.java:1480-1483,1502-1503 (V24.4 exemption so these pulls are 'NEVER penalize, always fire'); DeployPhaseScript.java:200-207 (qualify() empties character buckets on turn &lt;= 2 with no battleground)</t>
         </is>
       </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="147" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1130,6 +1201,11 @@
           <t>V156: CharacterDeploySiteEvaluator.java:462-527 (-600 at :517-519, ability&gt;=6 fall-through :515,:526); V38: DeployEvaluator.java:2292-2529 (gate :2300-2302, wouldBeSolo default :2317, -150 at :2516-2522); V113: CardSelectionEvaluator.java:2903-2927 (-300 at :2918-2926, ability&gt;=3 gate :2918); V29.5: CardSelectionEvaluator.java:2877-2901; V136 dual routes: DeployEvaluator.java:1759-1775 and CardSelectionEvaluator.java:2056-2072</t>
         </is>
       </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="147" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1192,6 +1268,11 @@
           <t>V156 exemption + turn gate: CharacterDeploySiteEvaluator.java:501-527 (currentTurn&lt;=2 gate :501, ability&gt;=6 :515); V137 ANTI-SOLO BG: MoveEvaluator.java:1060-1100 (no ability check, no turn check, -500 at :1093-1099); V137 header admitting the deploy/move contradiction class: MoveEvaluator.java:976-992</t>
         </is>
       </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="147" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1254,6 +1335,11 @@
           <t>V96 diff window incl. -10 and pre-deploy friendlyPower: DeployEvaluator.java:1862-1888 (+500 at :1872-1879); V136 §A losing tiers: CharacterDeploySiteEvaluator.java:529-536; V51 ungated drain bonuses: DeployEvaluator.java:2797-2842 (+600 :2805-2811, +500 :2812-2832); gated CS-side mirrors: CardSelectionEvaluator.java:879-908 (V177 survivability gate on V166), :1045-1076 (V172 winnability gate on V171)</t>
         </is>
       </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="147" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1316,6 +1402,11 @@
           <t>Block 1 (opp drain): DeployEvaluator.java:2797-2842 (+500 REINFORCE BATTLEGROUND :2826-2832; V36 drain-1 arm :2833-2841); Block 2 (our drain): DeployEvaluator.java:3176-3265 (+500 FORTIFY :3200-3206, +400 ESTABLISH :3207-3213, +300 REINFORCE :3214-3220, BUDDY tiers :3231-3252, +150 ARMED :3254-3263)</t>
         </is>
       </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="147" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1378,6 +1469,11 @@
           <t>DrawEvaluator.java:474-489 (no zone check on the opponent-card scan) vs PassEvaluator.java:190-196 (dtfZone.isInPlay()), MoveEvaluator.java:~405-412 (pZ.isInPlay() gate at loop top), DeployEvaluator.java:2258-2262 (dtfZ.isInPlay()), DeployEvaluator.java:2352-2358 (dtfChkZ.isInPlay())</t>
         </is>
       </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="147" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1440,6 +1536,11 @@
           <t>V85 block + return: MoveEvaluator.java:1721-1774 (return at 1768); V73 shuttle: MoveEvaluator.java:2137-2203 (comment claiming it beats V29.13 at 2142-2145); V29.13 drain-delta it was meant to beat: MoveEvaluator.java:2011-2063; call order: rankMoveFromLocation invoked at MoveEvaluator.java:469</t>
         </is>
       </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="147" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1502,6 +1603,11 @@
           <t>V85: MoveEvaluator.java:1739-1768 (no objective check, -2000); hunt trigger theirPowerHere==0: MoveEvaluator.java:920; V35 bonus +350: MoveEvaluator.java:958-967 + RandoConfig.java:182; V29.13 grouping +200/+250: MoveEvaluator.java:1170-1176, 1252-1257; V22.2 reinforce +80..160: MoveEvaluator.java:1411-1418</t>
         </is>
       </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="147" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1564,6 +1670,11 @@
           <t>V53b setScore(9999): MoveEvaluator.java:1606; V60 setScore(-9999): MoveEvaluator.java:1615; unprotected +800 Mapuzo-exit branch: MoveEvaluator.java:1622-1624; V37.1 -9999 stay blocks: MoveEvaluator.java:1697-1717; V85 -2000: MoveEvaluator.java:1758-1768; rankMoveFromLocation called first: MoveEvaluator.java:469; setScore replaces score: EvaluatedAction.java:105 (field :17, addReasoning :41)</t>
         </is>
       </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="147" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1626,6 +1737,11 @@
           <t>V137 canWin + penalties: MoveEvaluator.java:1047-1057 (thresholds :1047, -800/-1500 :1049-1050); V136 base thresholds: CharacterDeploySiteEvaluator.java:237-238; V181 fair-fight commit: CharacterDeploySiteEvaluator.java:334-385 (gap&lt;=3 :351, drain&gt;=2 :355, parity :372-373, +min(300, drain*100) :375); V137's origin story (fixing the V136-vs-V35 contradiction): MoveEvaluator.java:976-992</t>
         </is>
       </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="147" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1688,6 +1804,11 @@
           <t>V35.4 inverted detection + global +150/+250 boost: ActionTextEvaluator.java:3510-3548 (owner==us &amp;&amp; isUndercover -&gt; oppHasUndercoverSpy at :3525-3531, bonus :3538); V53 SPY STAY -300: MoveEvaluator.java:1557-1560; RETREAT tier that also pushes the spy out: MoveEvaluator.java:1686-1690; V170 deploy-side doctrine the spy is executing: CardSelectionEvaluator.java:968-994</t>
         </is>
       </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="147" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1750,6 +1871,11 @@
           <t>V47 lock + substring list: MoveEvaluator.java:362-381 ('platform' at :373, -9999 at :377); RETREAT tier +150: MoveEvaluator.java:1686-1690; V22.5 +100..160: MoveEvaluator.java:1324-1332; V53 spy-follow +500: MoveEvaluator.java:1553-1556</t>
         </is>
       </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="147" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1812,6 +1938,11 @@
           <t>Mirror block: CardSelectionEvaluator.java:4857-4946 (protections only at 4929-4943: objective-critical + priority card). Regular block protections: 3820-3851 (V109), 4045-4059 (V175/V175a), 4071-4096 (V178), 4144-4148 (V25), 4106-4127 (V28) — all live (verified uncommented), none present in 4857-4946</t>
         </is>
       </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="147" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1874,6 +2005,11 @@
           <t>DeployEvaluator.java:574-601 (fail-stop -9999 at 581-586, reserve&lt;=2 risk -9999 at 593-601, both with continue); ActionTextEvaluator.java:4264-4288 (reserve&lt;=2 risk -400 at 4269, fail-stop -9999 at 4282); DeployEvaluator.java:531-534 ('deploy'-word gate that decides which copy runs)</t>
         </is>
       </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="147" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1936,6 +2072,11 @@
           <t>DeployEvaluator.java:3331-3336 (V162 +500 + V67ai hand +1400 = +1900); DeployEvaluator.java:3434-3443 and ActionTextEvaluator.java:4697-4708 (V67ai pull tiers x2); ActionTextEvaluator.java:4243-4246 (V82 +2500); ActionTextEvaluator.java:1148-1151 (V100 +1500); ActionTextEvaluator.java:341-343 (V116 +100); DeployEvaluator.java:1084-1085 (V24.10 +150); DeployEvaluator.java:1118-1121 (V24.15 +400/+800); ActionTextEvaluator.java:1497-1499 (V24.4 -800); DeployPhaseScript.java:96-101 + CombinedEvaluator.java:109-138 (structural STEP 1 ordering); RandoCalAi.java:1130-1131 (DPS scope = CARD_ACTION_CHOICE only)</t>
         </is>
       </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="147" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1998,6 +2139,11 @@
           <t>DeployEvaluator.java:3320-3326 (V162 hold, -200 at life force &lt;= 10); ActionTextEvaluator.java:1448-1509 (V24.4: hasLocationInHand -&gt; -800 at 1497-1499, exemptions only for location-search/AMSD/reserve-pull/deploy-entry, no life-force check)</t>
         </is>
       </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="147" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -2060,6 +2206,11 @@
           <t>PassEvaluator.java:174-213 (V27.1 +20/40/60 at 201-207), PassEvaluator.java:215-251 (V27 +25/+50 at 238-246), PassEvaluator.java:146-148 (+8 small hand), 169-172 (+10 move phase); MoveEvaluator.java:383-462 (V29, -100/-150 at 448-456, -60 mild at 455)</t>
         </is>
       </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="147" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2122,6 +2273,11 @@
           <t>V85 engine-amount: MoveEvaluator.java:1741-1758; V29.13 engine-amount: MoveEvaluator.java:2035-2046; V67e icon-based: CardSelectionEvaluator.java:5913-5939; V67g move-from-drain icon-based: CardSelectionEvaluator.java:5993-6004; V67ae icon-based: ActionTextEvaluator.java:3482-3497; V63/V67d routing that decides which path fires: CardSelectionEvaluator.java:423-442</t>
         </is>
       </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="147" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -2184,6 +2340,11 @@
           <t>ShieldStrategy.java:461-485 (V105 power&gt;0 scan); CardSelectionEvaluator.java:7813-7841 (V112 char/ship/vehicle presence), 7847-7852 (-9999); CardSelectionEvaluator.java:8826-8851 (V51 any-owned-card presence), 8856-8858 (-9999); CardSelectionEvaluator.java:7892 + 7914-7917 (V117 boost keyed to prefers4thSlot)</t>
         </is>
       </c>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t>PARTIALLY-ADDRESSED (sev now low) by ee0a1b435 (predicate unification for V51/V112 + preferredShieldInCandidates), 8f841bd25 (V51 early-deploy rides on the unified predicate) — ee0a1b435 fixed 2 of the 3 divergent occupancy implementations: V112 (CardSelectionEvaluator.java:7819) and both V51 arms (8614, 8905) now share occupiesBothTheaters() (8729-8745, engine Filters.canSpot(occupies + battleground_site/system), matching the card's own condition), and preferredShieldInCandidates() (8759-8785, consumed at 7898 and 8866) removed the hard-block-spam deadlock by holding the slot when the pref</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="147" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2246,6 +2407,11 @@
           <t>CardSelectionEvaluator.java:3820-3851 (V109 -300, applied before zone scoring); CardSelectionEvaluator.java:3996-4022 (V153 tiers: hand char 700 when protectChars=false, Used 400, Reserve 300, Force pile 50)</t>
         </is>
       </c>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="147" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -2308,6 +2474,11 @@
           <t>CardSelectionEvaluator.java:4144-4148 (V25 -500, isHuntDownV + title contains 'lightsaber'); 4071-4096 (V178 -450, WEAPON + wielder + turn&gt;3 + protectChars); 4012 (hand junk 600), 4008 (hand char 100), 4019 (force pile 50 'ALWAYS last')</t>
         </is>
       </c>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="147" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2370,6 +2541,11 @@
           <t>ForceActivationEvaluator.java:85-91 (V42 activation log on V57/V61c logic) vs DrawEvaluator.java:185-195 (V42 EMERGENCY DRAW +200..600); DeployPhasePlanner.java:199-227 (V22.3 maintenance reserve) vs ActionTextEvaluator.java:3941-3946 (V22.3 MAINTENANCE pay-upkeep +150)</t>
         </is>
       </c>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="147" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -2432,6 +2608,11 @@
           <t>CardSelectionEvaluator.java:4005-4006 (dup 1000), 4099-4103 (hand floor -700 with no isDuplicate exclusion), 4015/4017 (Used 800, Reserve 400); mirror: 4903 (dup 1000), 4920-4926 (floor, same gap)</t>
         </is>
       </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="147" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -2490,6 +2671,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/ActionTextEvaluator.java:4056-4059 (+20 even), :4052-4055 (+60 marginal), :4020 (case-sensitive contains); BattleEvaluator.java:483-499 (marginal -50 at 491, even -100 at 495), :462-465 (favorable sets foundFavorableBattle; marginal does NOT), :167 (lowercased contains), :569-570 (-60 keyed to foundFavorableBattle)</t>
         </is>
       </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="147" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -2548,6 +2734,11 @@
           <t>RandoCalAi.java:747-758 (evaluator-first, fallback on null), :1980-1981 + RandoConfig.java:26 (chaos dead: nextInt(100)&lt;0), RandoCalAi.java:129 (ACTION_WEIGHTS 'force drain'=200), :1393-1411 (scoreControlAction +120 via RandoConfig.java:143, +20*controlledBGs), :1263-1266 (+40 behind), HeuristicAiBase.java:1668-1677 + :1694-1698 (scoreAction sums keyword table + phase bias 'force drain'=120), :350-351 (scoreAction + scoreActionContext summed per action); guards existing only in ActionTextEvaluator.java:5058-5311</t>
         </is>
       </c>
+      <c r="M33" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now medium) — None of the six post-audit commits touched RandoCalAi.java, RandoConfig.java, or HeuristicAiBase.java (confirmed via git log --name-only fcec408b9~1..HEAD), so the fallback brain's triple-additive drain scoring (200+120+120, +20/controlled BG, +40 behind, approx 440-500) and the unguarded "cancel" +40 (RandoCalAi.java:155, V52 block exists only at ActionTextEvaluator.java:3894-3897) survive at identical lines with id</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="147" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -2606,6 +2797,11 @@
           <t>ActionTextEvaluator.java:46-53 (catch-all canEvaluate), :56-73 (MULTIPLE_CHOICE whitelist); RandoCalAi.java:742-760 (routing: chaos else tryEvaluators else super.decide), :127-207 (keyword tables), :1222-1516 (scoreActionContext + phase scorers), :1518-1536 (weight getters); RandoConfig.java:26 (CHAOS_PERCENT=0), :113-116 + :146 + :149 (duplicate battle thresholds, pass penalty 200); CombinedEvaluator.java:243-250 (canHandle); DecisionContext.java:55 (noPass defaults true → PassEvaluator can't hijack MULTIPLE_CHOICE); HeuristicAiBase.java:29-31 + :48 + :351-391 (failed-search penalties only in pickActionChoice; private DecisionTracker), :167-223 (pickMultipleChoice: CHOICE_WEIGHTS + findPassIndex -200); ActionTextEvaluator.java:213-260 (V177 gate lives only on the ATE path)</t>
         </is>
       </c>
+      <c r="M34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STILL-VALID (sev now medium) — The finding survives unchanged: none of the six commits touched the routing files (git log fcec408b9^..HEAD over RandoCalAi.java, HeuristicAiBase.java, RandoConfig.java, CombinedEvaluator.java, DecisionContext.java returns empty). At HEAD: ATE canEvaluate still catch-alls ACTION_CHOICE/CARD_ACTION_CHOICE and whitelists only the same four MULTIPLE_CHOICE text patterns (ActionTextEvaluator.java:45-77); CHAOS_PERCENT=0 </t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="147" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -2664,6 +2860,11 @@
           <t>V31 -50 spread nudge: DeployEvaluator.java:4426-4432; V36 +250 (non-HuntDown): DeployEvaluator.java:4395-4425; V51 CC ARMY +500: DeployEvaluator.java:3595-3617; V51 OBJ FIRST +300: DeployEvaluator.java:3619-3642; V51 FORTIFY +500: DeployEvaluator.java:3200-3206; V38 REINFORCE +200..400: DeployEvaluator.java:2531-2576; V113 no objective exemption: CardSelectionEvaluator.java:2903-2927; V156's contrasting objective skip: CharacterDeploySiteEvaluator.java:501-502</t>
         </is>
       </c>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="147" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -2722,6 +2923,11 @@
           <t>V51 BUDDY DESTINY +400: DeployEvaluator.java:3231-3237 (literal 4.0f), BUDDY FULL +500 :3238-3244 (literal 7.0f); V32 ABILITY FIX +150: DeployEvaluator.java:4557-4566 (literal 4.0f); V38 REINFORCE ALLY +300: DeployEvaluator.java:2563-2571 (RandoConfig.ABILITY_BUDDY_THRESHOLD, RandoConfig.java:93 = 7); V136 §A abilityPass: CharacterDeploySiteEvaluator.java:238,:529; V32 lying log (0.0f added, log says -200): DeployEvaluator.java:4589-4595</t>
         </is>
       </c>
+      <c r="M36" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="147" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -2780,6 +2986,11 @@
           <t>DeployEvaluator.java:2029 (battleReserve=2), 2061-2081 (V59 -2000 / HOLISTIC -1500 / V64 -400), 2092-2133 (V24.5 -50 at 2117 and 2124), 2230-2245 (V29.13 -50/-500 at 2241), 2282 (V29.13 interrupt -30); DeployPhasePlanner.java:198-227 (V22.3 effectiveForce)</t>
         </is>
       </c>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="147" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -2842,6 +3053,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/BattleEvaluator.java:575-616 (must-fight +200 at 610-612), :429-441 (V76 -800 at 432, -500 at 438), :495 (even-or-worse -100), :570 (no-favorable -60), :140 (base 100)</t>
         </is>
       </c>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="147" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -2904,6 +3120,11 @@
           <t>DeployEvaluator.java:3369-3377 (V67i keyword list); ActionTextEvaluator.java:4510-4518 (V67l identical list); ActionTextEvaluator.java:4238-4240 (V82 regex nouns); ActionTextEvaluator.java:1108-1119 (V100 nouns) + 1131-1147 (char-in-hand gate); ActionTextEvaluator.java:4586-4589 (V131 locNouns, so 'farm' pulls skip deck-aware validation entirely at 4595-4632)</t>
         </is>
       </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="147" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -2966,6 +3187,11 @@
           <t>DeployPhasePlanner.java:227 (effectiveForce = forceAvailable - battleForceReserve - maintenanceReserve) with RandoConfig.java:46 (BATTLE_FORCE_RESERVE = 1); DeployEvaluator.java:2029 (battleReserve = 2); DeployEvaluator.java:935-977 (V176 -800 at pile &lt;= 2)</t>
         </is>
       </c>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="147" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -3028,6 +3254,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/BattleEvaluator.java:259-309 (Barrier -150 at 285, -250 at 286, -100 at 287, ×factor at 295), :311-327 (aggressiveness +80/+200 at 318-319), :329-379 (V35 destiny +120/+250/+100 at 366-368); RandoConfig.java:194 (VADER_EXPENDABILITY_FACTOR = 0.3f)</t>
         </is>
       </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="147" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -3090,6 +3321,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/BattleEvaluator.java:622-663 (V61 chain; V61b skip 632-644 wraps only this chain), :700-729 (V27.1 -100/-60 at 706-711, V27 -40 at 723, -15 at 727), :736-738 (ahead -20); ActionTextEvaluator.java:4083-4090 (V25 reserve -50, no overpower carve-out)</t>
         </is>
       </c>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="147" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -3152,6 +3388,11 @@
           <t>ActionTextEvaluator.java:5266-5273 (V140 waiver +VERY_GOOD_DELTA+10 then return), :5300-5311 (turn&gt;=3 paid path +50, no return), :5186-5191 (no-deployables +70 return), :5324-5368 (FIX 14 tiers only reachable when no early return), :5375-5399 (V29.9 also skipped on return)</t>
         </is>
       </c>
+      <c r="M43" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now low) — cb98f0075 fixed only the waiver DETECTION: v140CostWaived now fires solely when the engine says initiate-cost is 0 (getInitiateForceDrainCost at :5290-5291), so the finding's specific boundary premise ("Battle Plan on table = universal waiver") is stale. But the contradiction itself survives unchanged: a genuinely free drain (Rando occupies BG site + BG system) still scores a flat +60 and returns, skipping the FIX 14</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="147" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3214,6 +3455,11 @@
           <t>ActionTextEvaluator.java:3131-3139 (routing branch, earlier in the same if/else chain — no method boundary between 3100-3900 per awk scan), :3894-3901 (shadowed V52 copy A), :5430-5486 (evaluateSenseCancel; high-value branches :5461-5472 precede the V52 drain guard :5473-5480), AiPriorityCards.java:305/:324/:325 ('sense' 85, 'alter' 55, 'control' 55), :352-371 (substring matcher)</t>
         </is>
       </c>
+      <c r="M44" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="147" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -3276,6 +3522,11 @@
           <t>ActionTextEvaluator.java:107 (blocked entry), :144-147 (V167 -200, no continue), :160-187 (V168 +5000 at :186, V61c -6000 at :181); DecisionTracker.java:340-356 (getBlockedResponses feeding the set), :461 (turnBlockedActions written by blockLastActionOnCancel); PassEvaluator.java:85 (Pass ~5)</t>
         </is>
       </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="147" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -3338,6 +3589,11 @@
           <t>PassEvaluator.java:152-164 (V37.4 bloat penalty, DEPLOY only), :215-251 (V27 maintenance +25/+50, `!isActivateDecision` only), :174-213 (V27.1 DTF +20/40/60, not deploy-excluded), :85 (base 5), :139-141 (reserve&lt;10 +3)</t>
         </is>
       </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="147" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -3400,6 +3656,11 @@
           <t>DrawEvaluator.java:502 (maintenanceCost += 1), DrawEvaluator.java:432 (doc claims +N cost), DrawEvaluator.java:539 (added to reserve), DrawEvaluator.java:320-328 (DRAW-DOWN +80/surplus cap 400); vs PassEvaluator.java:232-234 (deployCost), DeployPhasePlanner.java:215-217 (deployCost), DeployEvaluator.java:2020-2023 (maintenanceCost = cost), DeployEvaluator.java:2107-2110 (deployCost)</t>
         </is>
       </c>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="147" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -3462,6 +3723,11 @@
           <t>CardSelectionEvaluator.java:8785 (shieldsRemaining()&lt;=1 gate), 8809-8811 (-5000 HOLD); CardSelectionEvaluator.java:7874-7885 (V117 table count &gt;=3), 7897-7901 (-9999); ActionTextEvaluator.java:2477-2500 (V124 table count), 2504 (-3000); ShieldStrategy.java:371-373 (shieldsRemaining), 606-607 (shieldsPlayed.add, never removed); RandoCalAi.java:1797-1802 (trackOwnShields populates tracker)</t>
         </is>
       </c>
+      <c r="M48" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now low) — The count-predicate split survives all six commits: V105/V107 still gates on the append-only shieldsPlayed tracker (ShieldStrategy.java:607 add, never removed, untouched since pre-audit 351a0523b) while V117 and V124 still do independent live table scans, with magnitude drift -5000/-9999/-3000 intact. Commit ee0a1b435 rewrote the logic INSIDE the V105 and V117 gates (preferredShieldInCandidates on-menu check, occupie</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="147" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -3524,6 +3790,11 @@
           <t>ShieldStrategy.java:765-769 (turnNumber &lt; 4 release), 843-852 (last-slot +50/-30/-40), 702 (design comment 'released on turn 4+'); CardSelectionEvaluator.java:8806-8814 (-5000 HOLD 'closed indefinitely'); CardSelectionEvaluator.java:7897-7901 (V117 -9999)</t>
         </is>
       </c>
+      <c r="M49" s="11" t="inlineStr">
+        <is>
+          <t>STILL-VALID (sev now low) — ShieldStrategy.java was not touched by any of the six commits (last change is the pre-audit 351a0523b snapshot), so the V29 turn-4 release (line 765), the last-slot +50/-30/-40 adjustments (~843-852), and the design comment (~702) are all still live. The ee0a1b435 rework of CardSelectionEvaluator changed the gate's mechanism (preferred-shield-on-menu check, HOLD path instead of per-card block spam, V117 twin fix at 7</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="147" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -3586,6 +3857,11 @@
           <t>ActionTextEvaluator.java:5445-5453 (V37.3 list + -9999 + return, no owner check); AiPriorityCards.java:297-298 (ghhhk=100 critical), 302 (sith fury 90); ActionTextEvaluator.java:5459-5472 (unreachable high-value cancel scoring for listed titles)</t>
         </is>
       </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="147" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -3648,6 +3924,11 @@
           <t>ActionTextEvaluator.java:3893-3901 (copy 1); 3132-3138 (earlier shadowing branch, same else-if chain — verified no method boundary between 3138 and 3894); 5461-5480 (copy 2: pattern branches checked before the isMyTurn drain guard at 5475); AiPriorityCards.java:305-306, 324-325 (pattern words)</t>
         </is>
       </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>unaffected — cited code untouched since audit base 8392f3868 (diff-checked 2026-07-06)</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="147" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
@@ -3710,6 +3991,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/BattleEvaluator.java:509 (fallback gate), :542-555 (V164a +40, fallback only), :493-499 (specific branch even-or-worse -100), :569-570 (-60), :163-171 (title match sets targetLocation)</t>
         </is>
       </c>
+      <c r="M52" s="12" t="inlineStr">
+        <is>
+          <t>refuted at audit — n/a</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="147" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
@@ -3772,6 +4058,11 @@
           <t>src/gemp-swccg-server/src/main/java/com/gempukku/swccgo/ai/models/rando/evaluators/ActionTextEvaluator.java:2589 (if contains 'hatred'), :2644-2647 (V35.7 -500 no Inquisitor), :2650-2651 (+400/+350 +150), :2723-2725 (if contains 'far more frightening'; USED mode = stack||hatred-without-destiny), :2764-2770 (FMFTD USED +350/+150, no Inquisitor check); RandoConfig.java:185 (SCORE_HATRED_WITH_INQUISITOR=400)</t>
         </is>
       </c>
+      <c r="M53" s="12" t="inlineStr">
+        <is>
+          <t>refuted at audit — n/a</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="147" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
@@ -3834,6 +4125,11 @@
           <t>PassEvaluator.java:25-27 (CANCEL_KEYWORDS incl. 'cancel'), :64-83 (substitution), :126-251 (conservation bonuses attached to the substituted id), :266-305 (findCancelAction); ActionTextEvaluator.java:46-53 (ATE scores every ACTION_CHOICE action), :3893-3900 (drain-cancel +30 / -9999); CombinedEvaluator.java:71-86 (same-id merge)</t>
         </is>
       </c>
+      <c r="M54" s="12" t="inlineStr">
+        <is>
+          <t>refuted at audit — n/a</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="147" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
@@ -3894,6 +4190,11 @@
       <c r="L55" s="6" t="inlineStr">
         <is>
           <t>V37 -800: MoveEvaluator.java:813-820; V137 ANTI-SOLO-BG -500: MoveEvaluator.java:1093-1099 (projected count :1092); RETREAT tier +150 (VERY_GOOD_DELTA): MoveEvaluator.java:1686-1690 + :54; V22.5 +60..160: MoveEvaluator.java:1305-1337; V169 destination-step-only fix: CardSelectionEvaluator.java:5751-5782 and +600 at :5867-5872</t>
+        </is>
+      </c>
+      <c r="M55" s="12" t="inlineStr">
+        <is>
+          <t>refuted at audit — n/a</t>
         </is>
       </c>
     </row>
@@ -3909,7 +4210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3996,6 +4297,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>T0.0 reconcile (2026-07-06)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>9 findings re-verified at HEAD 8f841bd25 after V177/V189/V190/V51-V105-V112-V117 in-place fixes: 2 partially addressed (control-drain-1 by V189; shields-response-2 by ee0a1b435), 7 still valid (control-drain-5 and deploy-sequencing-1 remain HIGH; control-drain-4 gap WIDENED: V189 protections are evaluator-brain only). Remaining 41 non-refuted rows: cited code untouched (diff-checked).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>